<commit_message>
Atualiza relatório volume 3 com dados de agosto
</commit_message>
<xml_diff>
--- a/public/data/predilecta_banco_dados_com_caminhoes.xlsx
+++ b/public/data/predilecta_banco_dados_com_caminhoes.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultado" sheetId="1" r:id="R12b07496e94343d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolução" sheetId="2" r:id="Rcd172babf1324ff4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caminhoes" sheetId="3" r:id="Rfae6a25991af4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultado" sheetId="1" r:id="Rc7ffcf8c936f424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolução" sheetId="2" r:id="R8e90a06241124f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caminhoes" sheetId="3" r:id="Rc35d5918035e40fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -71,7 +71,6 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -80,7 +79,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultadoTable" displayName="ResultadoTable" ref="A1:D85" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultadoTable" displayName="ResultadoTable" ref="A1:D57" headerRowCount="1">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Mês"/>
     <x:tableColumn id="2" name="Transportadora"/>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvolucaoTable" displayName="EvolucaoTable" ref="A1:D245" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EvolucaoTable" displayName="EvolucaoTable" ref="A1:D121" headerRowCount="1">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Data"/>
     <x:tableColumn id="2" name="Transportadora"/>
@@ -1073,402 +1072,10 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B58" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C58" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D58" t="n">
-        <x:v>503</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B59" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C59" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D59" t="n">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B60" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C60" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D60" t="n">
-        <x:v>240</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B61" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C61" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D61" t="n">
-        <x:v>49</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B62" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C62" t="str">
-        <x:v>SóFruta</x:v>
-      </x:c>
-      <x:c r="D62" t="n">
-        <x:v>242</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B63" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C63" t="str">
-        <x:v>SóFruta</x:v>
-      </x:c>
-      <x:c r="D63" t="n">
-        <x:v>27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B64" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C64" t="str">
-        <x:v>SóFruta</x:v>
-      </x:c>
-      <x:c r="D64" t="n">
-        <x:v>147</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B65" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C65" t="str">
-        <x:v>SóFruta</x:v>
-      </x:c>
-      <x:c r="D65" t="n">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B66" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C66" t="str">
-        <x:v>StellaDóro</x:v>
-      </x:c>
-      <x:c r="D66" t="n">
-        <x:v>254</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B67" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C67" t="str">
-        <x:v>StellaDóro</x:v>
-      </x:c>
-      <x:c r="D67" t="n">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B68" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C68" t="str">
-        <x:v>StellaDóro</x:v>
-      </x:c>
-      <x:c r="D68" t="n">
-        <x:v>87</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B69" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C69" t="str">
-        <x:v>StellaDóro</x:v>
-      </x:c>
-      <x:c r="D69" t="n">
-        <x:v>22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B70" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C70" t="str">
-        <x:v>Minas+</x:v>
-      </x:c>
-      <x:c r="D70" t="n">
-        <x:v>186</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B71" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C71" t="str">
-        <x:v>Minas+</x:v>
-      </x:c>
-      <x:c r="D71" t="n">
-        <x:v>55</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B72" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C72" t="str">
-        <x:v>Minas+</x:v>
-      </x:c>
-      <x:c r="D72" t="n">
-        <x:v>174</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B73" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C73" t="str">
-        <x:v>Minas+</x:v>
-      </x:c>
-      <x:c r="D73" t="n">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74">
-      <x:c r="A74" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B74" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C74" t="str">
-        <x:v>Salsaretti</x:v>
-      </x:c>
-      <x:c r="D74" t="n">
-        <x:v>122</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75">
-      <x:c r="A75" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B75" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C75" t="str">
-        <x:v>Salsaretti</x:v>
-      </x:c>
-      <x:c r="D75" t="n">
-        <x:v>39</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76">
-      <x:c r="A76" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B76" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C76" t="str">
-        <x:v>Salsaretti</x:v>
-      </x:c>
-      <x:c r="D76" t="n">
-        <x:v>85</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77">
-      <x:c r="A77" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B77" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C77" t="str">
-        <x:v>Salsaretti</x:v>
-      </x:c>
-      <x:c r="D77" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78">
-      <x:c r="A78" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B78" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C78" t="str">
-        <x:v>Nordeste</x:v>
-      </x:c>
-      <x:c r="D78" t="n">
-        <x:v>37</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79">
-      <x:c r="A79" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B79" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C79" t="str">
-        <x:v>Nordeste</x:v>
-      </x:c>
-      <x:c r="D79" t="n">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80">
-      <x:c r="A80" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B80" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C80" t="str">
-        <x:v>Nordeste</x:v>
-      </x:c>
-      <x:c r="D80" t="n">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81">
-      <x:c r="A81" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B81" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C81" t="str">
-        <x:v>Nordeste</x:v>
-      </x:c>
-      <x:c r="D81" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B82" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C82" t="str">
-        <x:v>Goiás</x:v>
-      </x:c>
-      <x:c r="D82" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B83" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C83" t="str">
-        <x:v>Goiás</x:v>
-      </x:c>
-      <x:c r="D83" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B84" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C84" t="str">
-        <x:v>Goiás</x:v>
-      </x:c>
-      <x:c r="D84" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B85" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C85" t="str">
-        <x:v>Goiás</x:v>
-      </x:c>
-      <x:c r="D85" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7147f716fa3c48b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35594440eacb4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3177,1746 +2784,10 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="122">
-      <x:c r="A122" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B122" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C122" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D122" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123">
-      <x:c r="A123" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B123" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C123" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D123" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124">
-      <x:c r="A124" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B124" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C124" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D124" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="125">
-      <x:c r="A125" s="10" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B125" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C125" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D125" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126">
-      <x:c r="A126" s="10" t="n">
-        <x:v>46205</x:v>
-      </x:c>
-      <x:c r="B126" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C126" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D126" t="n">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="127">
-      <x:c r="A127" s="10" t="n">
-        <x:v>46205</x:v>
-      </x:c>
-      <x:c r="B127" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C127" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D127" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="128">
-      <x:c r="A128" s="10" t="n">
-        <x:v>46205</x:v>
-      </x:c>
-      <x:c r="B128" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C128" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D128" t="n">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="129">
-      <x:c r="A129" s="10" t="n">
-        <x:v>46205</x:v>
-      </x:c>
-      <x:c r="B129" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C129" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D129" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="130">
-      <x:c r="A130" s="10" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="B130" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C130" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D130" t="n">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="131">
-      <x:c r="A131" s="10" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="B131" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C131" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D131" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="132">
-      <x:c r="A132" s="10" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="B132" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C132" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D132" t="n">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="133">
-      <x:c r="A133" s="10" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="B133" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C133" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D133" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="134">
-      <x:c r="A134" s="10" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="B134" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C134" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D134" t="n">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="135">
-      <x:c r="A135" s="10" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="B135" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C135" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D135" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="136">
-      <x:c r="A136" s="10" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="B136" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C136" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D136" t="n">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137">
-      <x:c r="A137" s="10" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="B137" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C137" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D137" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="138">
-      <x:c r="A138" s="10" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="B138" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C138" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D138" t="n">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="139">
-      <x:c r="A139" s="10" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="B139" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C139" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D139" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="140">
-      <x:c r="A140" s="10" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="B140" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C140" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D140" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="141">
-      <x:c r="A141" s="10" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="B141" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C141" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D141" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="142">
-      <x:c r="A142" s="10" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="B142" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C142" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D142" t="n">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="143">
-      <x:c r="A143" s="10" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="B143" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C143" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D143" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="144">
-      <x:c r="A144" s="10" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="B144" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C144" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D144" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="145">
-      <x:c r="A145" s="10" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="B145" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C145" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D145" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="146">
-      <x:c r="A146" s="10" t="n">
-        <x:v>46210</x:v>
-      </x:c>
-      <x:c r="B146" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C146" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D146" t="n">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="147">
-      <x:c r="A147" s="10" t="n">
-        <x:v>46210</x:v>
-      </x:c>
-      <x:c r="B147" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C147" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D147" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="148">
-      <x:c r="A148" s="10" t="n">
-        <x:v>46210</x:v>
-      </x:c>
-      <x:c r="B148" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C148" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D148" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="149">
-      <x:c r="A149" s="10" t="n">
-        <x:v>46210</x:v>
-      </x:c>
-      <x:c r="B149" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C149" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D149" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="150">
-      <x:c r="A150" s="10" t="n">
-        <x:v>46211</x:v>
-      </x:c>
-      <x:c r="B150" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C150" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D150" t="n">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="151">
-      <x:c r="A151" s="10" t="n">
-        <x:v>46211</x:v>
-      </x:c>
-      <x:c r="B151" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C151" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D151" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="152">
-      <x:c r="A152" s="10" t="n">
-        <x:v>46211</x:v>
-      </x:c>
-      <x:c r="B152" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C152" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D152" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="153">
-      <x:c r="A153" s="10" t="n">
-        <x:v>46211</x:v>
-      </x:c>
-      <x:c r="B153" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C153" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D153" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="154">
-      <x:c r="A154" s="10" t="n">
-        <x:v>46212</x:v>
-      </x:c>
-      <x:c r="B154" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C154" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D154" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="155">
-      <x:c r="A155" s="10" t="n">
-        <x:v>46212</x:v>
-      </x:c>
-      <x:c r="B155" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C155" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D155" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="156">
-      <x:c r="A156" s="10" t="n">
-        <x:v>46212</x:v>
-      </x:c>
-      <x:c r="B156" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C156" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D156" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="157">
-      <x:c r="A157" s="10" t="n">
-        <x:v>46212</x:v>
-      </x:c>
-      <x:c r="B157" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C157" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D157" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="158">
-      <x:c r="A158" s="10" t="n">
-        <x:v>46213</x:v>
-      </x:c>
-      <x:c r="B158" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C158" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D158" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159">
-      <x:c r="A159" s="10" t="n">
-        <x:v>46213</x:v>
-      </x:c>
-      <x:c r="B159" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C159" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D159" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="160">
-      <x:c r="A160" s="10" t="n">
-        <x:v>46213</x:v>
-      </x:c>
-      <x:c r="B160" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C160" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D160" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="161">
-      <x:c r="A161" s="10" t="n">
-        <x:v>46213</x:v>
-      </x:c>
-      <x:c r="B161" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C161" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D161" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162">
-      <x:c r="A162" s="10" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B162" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C162" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D162" t="n">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="163">
-      <x:c r="A163" s="10" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B163" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C163" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D163" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="164">
-      <x:c r="A164" s="10" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B164" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C164" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D164" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="165">
-      <x:c r="A165" s="10" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B165" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C165" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D165" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="166">
-      <x:c r="A166" s="10" t="n">
-        <x:v>46215</x:v>
-      </x:c>
-      <x:c r="B166" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C166" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D166" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="167">
-      <x:c r="A167" s="10" t="n">
-        <x:v>46215</x:v>
-      </x:c>
-      <x:c r="B167" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C167" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D167" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="168">
-      <x:c r="A168" s="10" t="n">
-        <x:v>46215</x:v>
-      </x:c>
-      <x:c r="B168" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C168" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D168" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="169">
-      <x:c r="A169" s="10" t="n">
-        <x:v>46215</x:v>
-      </x:c>
-      <x:c r="B169" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C169" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D169" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="170">
-      <x:c r="A170" s="10" t="n">
-        <x:v>46216</x:v>
-      </x:c>
-      <x:c r="B170" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C170" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D170" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="171">
-      <x:c r="A171" s="10" t="n">
-        <x:v>46216</x:v>
-      </x:c>
-      <x:c r="B171" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C171" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D171" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="172">
-      <x:c r="A172" s="10" t="n">
-        <x:v>46216</x:v>
-      </x:c>
-      <x:c r="B172" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C172" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D172" t="n">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="173">
-      <x:c r="A173" s="10" t="n">
-        <x:v>46216</x:v>
-      </x:c>
-      <x:c r="B173" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C173" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D173" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="174">
-      <x:c r="A174" s="10" t="n">
-        <x:v>46217</x:v>
-      </x:c>
-      <x:c r="B174" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C174" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D174" t="n">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="175">
-      <x:c r="A175" s="10" t="n">
-        <x:v>46217</x:v>
-      </x:c>
-      <x:c r="B175" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C175" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D175" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="176">
-      <x:c r="A176" s="10" t="n">
-        <x:v>46217</x:v>
-      </x:c>
-      <x:c r="B176" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C176" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D176" t="n">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="177">
-      <x:c r="A177" s="10" t="n">
-        <x:v>46217</x:v>
-      </x:c>
-      <x:c r="B177" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C177" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D177" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="178">
-      <x:c r="A178" s="10" t="n">
-        <x:v>46218</x:v>
-      </x:c>
-      <x:c r="B178" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C178" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D178" t="n">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="179">
-      <x:c r="A179" s="10" t="n">
-        <x:v>46218</x:v>
-      </x:c>
-      <x:c r="B179" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C179" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D179" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="180">
-      <x:c r="A180" s="10" t="n">
-        <x:v>46218</x:v>
-      </x:c>
-      <x:c r="B180" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C180" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D180" t="n">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="181">
-      <x:c r="A181" s="10" t="n">
-        <x:v>46218</x:v>
-      </x:c>
-      <x:c r="B181" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C181" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D181" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="182">
-      <x:c r="A182" s="10" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="B182" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C182" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D182" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="183">
-      <x:c r="A183" s="10" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="B183" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C183" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D183" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="184">
-      <x:c r="A184" s="10" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="B184" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C184" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D184" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="185">
-      <x:c r="A185" s="10" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="B185" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C185" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D185" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="186">
-      <x:c r="A186" s="10" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="B186" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C186" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D186" t="n">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="187">
-      <x:c r="A187" s="10" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="B187" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C187" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D187" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="188">
-      <x:c r="A188" s="10" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="B188" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C188" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D188" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="189">
-      <x:c r="A189" s="10" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="B189" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C189" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D189" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="190">
-      <x:c r="A190" s="10" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="B190" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C190" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D190" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="191">
-      <x:c r="A191" s="10" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="B191" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C191" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D191" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="192">
-      <x:c r="A192" s="10" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="B192" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C192" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D192" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="193">
-      <x:c r="A193" s="10" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="B193" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C193" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D193" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="194">
-      <x:c r="A194" s="10" t="n">
-        <x:v>46222</x:v>
-      </x:c>
-      <x:c r="B194" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C194" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D194" t="n">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="195">
-      <x:c r="A195" s="10" t="n">
-        <x:v>46222</x:v>
-      </x:c>
-      <x:c r="B195" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C195" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D195" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="196">
-      <x:c r="A196" s="10" t="n">
-        <x:v>46222</x:v>
-      </x:c>
-      <x:c r="B196" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C196" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D196" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="197">
-      <x:c r="A197" s="10" t="n">
-        <x:v>46222</x:v>
-      </x:c>
-      <x:c r="B197" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C197" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D197" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="198">
-      <x:c r="A198" s="10" t="n">
-        <x:v>46223</x:v>
-      </x:c>
-      <x:c r="B198" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C198" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D198" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="199">
-      <x:c r="A199" s="10" t="n">
-        <x:v>46223</x:v>
-      </x:c>
-      <x:c r="B199" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C199" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D199" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="200">
-      <x:c r="A200" s="10" t="n">
-        <x:v>46223</x:v>
-      </x:c>
-      <x:c r="B200" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C200" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D200" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="201">
-      <x:c r="A201" s="10" t="n">
-        <x:v>46223</x:v>
-      </x:c>
-      <x:c r="B201" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C201" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D201" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="202">
-      <x:c r="A202" s="10" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B202" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C202" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D202" t="n">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="203">
-      <x:c r="A203" s="10" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B203" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C203" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D203" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="204">
-      <x:c r="A204" s="10" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B204" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C204" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D204" t="n">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="205">
-      <x:c r="A205" s="10" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B205" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C205" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D205" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="206">
-      <x:c r="A206" s="10" t="n">
-        <x:v>46225</x:v>
-      </x:c>
-      <x:c r="B206" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C206" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D206" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="207">
-      <x:c r="A207" s="10" t="n">
-        <x:v>46225</x:v>
-      </x:c>
-      <x:c r="B207" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C207" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D207" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="208">
-      <x:c r="A208" s="10" t="n">
-        <x:v>46225</x:v>
-      </x:c>
-      <x:c r="B208" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C208" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D208" t="n">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="209">
-      <x:c r="A209" s="10" t="n">
-        <x:v>46225</x:v>
-      </x:c>
-      <x:c r="B209" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C209" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D209" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="210">
-      <x:c r="A210" s="10" t="n">
-        <x:v>46226</x:v>
-      </x:c>
-      <x:c r="B210" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C210" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D210" t="n">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="211">
-      <x:c r="A211" s="10" t="n">
-        <x:v>46226</x:v>
-      </x:c>
-      <x:c r="B211" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C211" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D211" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="212">
-      <x:c r="A212" s="10" t="n">
-        <x:v>46226</x:v>
-      </x:c>
-      <x:c r="B212" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C212" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D212" t="n">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="213">
-      <x:c r="A213" s="10" t="n">
-        <x:v>46226</x:v>
-      </x:c>
-      <x:c r="B213" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C213" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D213" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="214">
-      <x:c r="A214" s="10" t="n">
-        <x:v>46227</x:v>
-      </x:c>
-      <x:c r="B214" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C214" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D214" t="n">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="215">
-      <x:c r="A215" s="10" t="n">
-        <x:v>46227</x:v>
-      </x:c>
-      <x:c r="B215" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C215" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D215" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="216">
-      <x:c r="A216" s="10" t="n">
-        <x:v>46227</x:v>
-      </x:c>
-      <x:c r="B216" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C216" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D216" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="217">
-      <x:c r="A217" s="10" t="n">
-        <x:v>46227</x:v>
-      </x:c>
-      <x:c r="B217" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C217" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D217" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="218">
-      <x:c r="A218" s="10" t="n">
-        <x:v>46228</x:v>
-      </x:c>
-      <x:c r="B218" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C218" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D218" t="n">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="219">
-      <x:c r="A219" s="10" t="n">
-        <x:v>46228</x:v>
-      </x:c>
-      <x:c r="B219" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C219" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D219" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="220">
-      <x:c r="A220" s="10" t="n">
-        <x:v>46228</x:v>
-      </x:c>
-      <x:c r="B220" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C220" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D220" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="221">
-      <x:c r="A221" s="10" t="n">
-        <x:v>46228</x:v>
-      </x:c>
-      <x:c r="B221" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C221" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D221" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="222">
-      <x:c r="A222" s="10" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B222" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C222" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D222" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="223">
-      <x:c r="A223" s="10" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B223" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C223" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D223" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="224">
-      <x:c r="A224" s="10" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B224" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C224" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D224" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="225">
-      <x:c r="A225" s="10" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B225" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C225" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D225" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="226">
-      <x:c r="A226" s="10" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="B226" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C226" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D226" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="227">
-      <x:c r="A227" s="10" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="B227" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C227" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D227" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="228">
-      <x:c r="A228" s="10" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="B228" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C228" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D228" t="n">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="229">
-      <x:c r="A229" s="10" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="B229" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C229" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D229" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="230">
-      <x:c r="A230" s="10" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="B230" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C230" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D230" t="n">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="231">
-      <x:c r="A231" s="10" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="B231" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C231" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D231" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="232">
-      <x:c r="A232" s="10" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="B232" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C232" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D232" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="233">
-      <x:c r="A233" s="10" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="B233" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C233" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D233" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="234">
-      <x:c r="A234" s="10" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="B234" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C234" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D234" t="n">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="235">
-      <x:c r="A235" s="10" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="B235" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C235" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D235" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="236">
-      <x:c r="A236" s="10" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="B236" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C236" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D236" t="n">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="237">
-      <x:c r="A237" s="10" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="B237" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C237" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D237" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="238">
-      <x:c r="A238" s="10" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="B238" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C238" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D238" t="n">
-        <x:v>18</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="239">
-      <x:c r="A239" s="10" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="B239" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C239" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D239" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="240">
-      <x:c r="A240" s="10" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="B240" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C240" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D240" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="241">
-      <x:c r="A241" s="10" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="B241" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C241" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D241" t="n">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="242">
-      <x:c r="A242" s="10" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="B242" t="str">
-        <x:v>Frota</x:v>
-      </x:c>
-      <x:c r="C242" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D242" t="n">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="243">
-      <x:c r="A243" s="10" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="B243" t="str">
-        <x:v>Transpredi</x:v>
-      </x:c>
-      <x:c r="C243" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D243" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="244">
-      <x:c r="A244" s="10" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="B244" t="str">
-        <x:v>Terceiro</x:v>
-      </x:c>
-      <x:c r="C244" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D244" t="n">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="245">
-      <x:c r="A245" s="10" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="B245" t="str">
-        <x:v>FOB</x:v>
-      </x:c>
-      <x:c r="C245" t="str">
-        <x:v>Predilecta</x:v>
-      </x:c>
-      <x:c r="D245" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35459aacb80d49d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d14ffb7d97b444b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14625,7 +12496,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37501e5c71ca4ec2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b774ac63db148bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>